<commit_message>
Fixing up GL Account
</commit_message>
<xml_diff>
--- a/documentation/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/historical_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA9A7A5-A7CA-F045-ACED-36F1F6D6994E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7955B68B-B0DB-684F-96C2-A848DA9FCA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="1500" windowWidth="26960" windowHeight="15940" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="80">
   <si>
     <t>PaymentTerms</t>
   </si>
@@ -270,6 +270,12 @@
   </si>
   <si>
     <t>entryno, vendorno, company</t>
+  </si>
+  <si>
+    <t>no, name, company, source_system</t>
+  </si>
+  <si>
+    <t>no, name</t>
   </si>
 </sst>
 </file>
@@ -814,10 +820,10 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Fixing GL Account Source Key
</commit_message>
<xml_diff>
--- a/documentation/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/historical_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7955B68B-B0DB-684F-96C2-A848DA9FCA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B43A7BF-BE7B-F44C-AA45-ED4DDE97D0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="1500" windowWidth="26960" windowHeight="15940" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
@@ -817,7 +817,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
fix pipeline for shortcutdiemnsion1code
</commit_message>
<xml_diff>
--- a/documentation/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/historical_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E469CD-2ADF-1D4C-932B-227778ED93A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643C2F7B-3DF2-3F4A-A3FE-8589FBD87526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-260" yWindow="-19060" windowWidth="26960" windowHeight="15940" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
@@ -249,9 +249,6 @@
   </si>
   <si>
     <t>itemno, entrytype, sourceno, locationcode,  globaldimension1code, globaldimension2code,  shptmethodcode, sourcetype, itemtracking, packageno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">documenttype, selltocustomerno, billtocustomerno, billtocity,  shiptocity, paymenttermscode, shipmentmethodcode, locationcode,  shortcutdimension1code shortcutdimension2code, customerpostinggroup,  currencycode, customerpricegroup,  customerdiscgroup, languagecode, salespersoncode, genbuspostinggroup,  transactiontype, transportmethod,  vatcountryregioncode, selltocity,  billtopostcode, billtocounty, billtocountryregioncode, selltopostcode, selltocounty, selltocountryregioncode,  balaccounttype,  prepmtpaymenttermscode, selltocontactno, billtocontactno,  responsibilitycenter,  shippingadvice </t>
   </si>
   <si>
     <t>documenttype, selltocustomerno, no,  type,  locationcode, postinggroup, unitofmeasure,  shortcutdimension1code, shortcutdimension2code, customerpricegroup,  billtocustomerno,  purchaseorderno,  genbuspostinggroup,  genprodpostinggroup, vatcalculationtype,  transactiontype,  transportmethod,  taxcategory, vatbuspostinggroup, vatprodpostinggroup, currencycode, vatidentifier, prepmtvatcalctype, dimensionsetid, bincode, unitofmeasure,  itemcategorycode,  shippingagentcode,  shippingagentservicecode</t>
@@ -349,6 +346,9 @@
   </si>
   <si>
     <t>baseunitofmeasure,  type, inventorypostinggroup, shelfno, itemdiscgroup, vendorno, countryregionpurchasedcode,  globaldimension1code, globaldimension2code, flushingmethod,  salesunitofmeasure,  reorderingpolicy, manufacturingpolicy, itemcategorycode,  itemtrackingcode, subscriptionoption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">documenttype, selltocustomerno, billtocustomerno, billtocity,  shiptocity, paymenttermscode, shipmentmethodcode, locationcode,  shortcutdimension1code, shortcutdimension2code, customerpostinggroup,  currencycode, customerpricegroup,  customerdiscgroup, languagecode, salespersoncode, genbuspostinggroup,  transactiontype, transportmethod,  vatcountryregioncode, selltocity,  billtopostcode, billtocounty, billtocountryregioncode, selltopostcode, selltocounty, selltocountryregioncode,  balaccounttype,  prepmtpaymenttermscode, selltocontactno, billtocontactno,  responsibilitycenter,  shippingadvice </t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1032,7 @@
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F12" t="s">
         <v>63</v>
@@ -1072,7 +1072,7 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F14" t="s">
         <v>65</v>
@@ -1092,7 +1092,7 @@
         <v>51</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
         <v>61</v>
@@ -1112,7 +1112,7 @@
         <v>29</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>66</v>
@@ -1152,7 +1152,7 @@
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F18" t="s">
         <v>65</v>
@@ -1172,7 +1172,7 @@
         <v>51</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F19" t="s">
         <v>68</v>
@@ -1192,7 +1192,7 @@
         <v>29</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F20" t="s">
         <v>66</v>
@@ -1212,7 +1212,7 @@
         <v>51</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F21" t="s">
         <v>68</v>

</xml_diff>